<commit_message>
Dealer programme: staging second pass results (20 pass, D-2 fixed, D-3 open); report and tracker updated
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/dealer-programme/DEALER_PROGRAMME_TRACKER_2026-10-28.xlsx
+++ b/docs/dealer-programme/DEALER_PROGRAMME_TRACKER_2026-10-28.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="128">
   <si>
     <t>ID</t>
   </si>
@@ -71,7 +71,7 @@
     <t>PASS</t>
   </si>
   <si>
-    <t>PARTIAL — admin, geo PASS; operator check blocked</t>
+    <t>PASS — incl. operator refused</t>
   </si>
   <si>
     <t>Not released (flags off)</t>
@@ -110,7 +110,7 @@
     <t>3d92aaf</t>
   </si>
   <si>
-    <t>BLOCKED — no applicant account</t>
+    <t>PASS — application with documents</t>
   </si>
   <si>
     <t>GKS-DR-002</t>
@@ -122,7 +122,7 @@
     <t>Configurable document requirements; admin approval queue; suspend / reject / terminate</t>
   </si>
   <si>
-    <t>PARTIAL — D-1 fixed (f588580); approval blocked</t>
+    <t>PASS — approval; D-1 fixed</t>
   </si>
   <si>
     <t>GKS-DR-003</t>
@@ -134,7 +134,7 @@
     <t>GKS-MH-&lt;district&gt;-code, share link /shop/register?ref=, QR, suspend / replace</t>
   </si>
   <si>
-    <t>BLOCKED — no dealer</t>
+    <t>PASS — code, link, QR</t>
   </si>
   <si>
     <t>GKS-DR-004</t>
@@ -146,6 +146,9 @@
     <t>Salespeople with optional Employee ID; legacy distributors migrated as dealers</t>
   </si>
   <si>
+    <t>PASS — employee E01</t>
+  </si>
+  <si>
     <t>GKS-SH-001</t>
   </si>
   <si>
@@ -173,6 +176,9 @@
     <t>Dealer registers with the owner; owner confirms with a code</t>
   </si>
   <si>
+    <t>PASS — owner code by e-mail</t>
+  </si>
+  <si>
     <t>GKS-SH-003</t>
   </si>
   <si>
@@ -182,6 +188,9 @@
     <t>Phone / GSTIN / name within 150 m flagged; no commission</t>
   </si>
   <si>
+    <t>PARTIAL — automated tests only</t>
+  </si>
+  <si>
     <t>GKS-RA-001</t>
   </si>
   <si>
@@ -191,7 +200,7 @@
     <t>30-day leads (cap 200), attribution priority, dealer claims decided by staff</t>
   </si>
   <si>
-    <t>PARTIAL — claims page loads</t>
+    <t>PASS — lead, attribution</t>
   </si>
   <si>
     <t>GKS-SH-004</t>
@@ -209,7 +218,7 @@
     <t>4500808, 6db91cd</t>
   </si>
   <si>
-    <t>PARTIAL — page loads; approval needs owner + sandbox pay</t>
+    <t>FAIL — D-2 fixed in code, D-3 open</t>
   </si>
   <si>
     <t>GKS-CM-001</t>
@@ -227,7 +236,7 @@
     <t>22a74db</t>
   </si>
   <si>
-    <t>PARTIAL — rules visible; operator 403 blocked</t>
+    <t>PASS — rates; operator 403</t>
   </si>
   <si>
     <t>GKS-CM-002</t>
@@ -242,6 +251,9 @@
     <t>22a74db, 9e3e1b7</t>
   </si>
   <si>
+    <t>FAIL — no accrual on staging (D-3)</t>
+  </si>
+  <si>
     <t>GKS-CM-003</t>
   </si>
   <si>
@@ -251,7 +263,7 @@
     <t>Rating 0–10 by live shops (slabs), start rating, downgrade, bonus</t>
   </si>
   <si>
-    <t>PARTIAL — slabs visible</t>
+    <t>PARTIAL — slabs visible; no accrual yet</t>
   </si>
   <si>
     <t>GKS-DB-001</t>
@@ -266,6 +278,9 @@
     <t>89f66b9, c9ea939</t>
   </si>
   <si>
+    <t>PASS — board, phone width</t>
+  </si>
+  <si>
     <t>GKS-SP-001</t>
   </si>
   <si>
@@ -281,7 +296,7 @@
     <t>c70e869</t>
   </si>
   <si>
-    <t>PARTIAL — admin page; shop side blocked</t>
+    <t>PASS — free, wallet, refund, online</t>
   </si>
   <si>
     <t>GKS-GEO-001</t>
@@ -403,7 +418,7 @@
       <b/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -425,6 +440,11 @@
         <fgColor rgb="FFFEF3C7"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFEE2E2"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -438,7 +458,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -450,6 +470,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -869,7 +892,7 @@
       <c r="I2" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="J2" s="4" t="s">
+      <c r="J2" s="3" t="s">
         <v>19</v>
       </c>
       <c r="K2" s="2" t="s">
@@ -939,7 +962,7 @@
       <c r="I4" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="J4" s="4" t="s">
+      <c r="J4" s="3" t="s">
         <v>32</v>
       </c>
       <c r="K4" s="2" t="s">
@@ -974,7 +997,7 @@
       <c r="I5" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="J5" s="4" t="s">
+      <c r="J5" s="3" t="s">
         <v>36</v>
       </c>
       <c r="K5" s="2" t="s">
@@ -1009,7 +1032,7 @@
       <c r="I6" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="J6" s="4" t="s">
+      <c r="J6" s="3" t="s">
         <v>40</v>
       </c>
       <c r="K6" s="2" t="s">
@@ -1044,8 +1067,8 @@
       <c r="I7" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="J7" s="4" t="s">
-        <v>40</v>
+      <c r="J7" s="3" t="s">
+        <v>44</v>
       </c>
       <c r="K7" s="2" t="s">
         <v>20</v>
@@ -1053,13 +1076,13 @@
     </row>
     <row r="8" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>14</v>
@@ -1068,10 +1091,10 @@
         <v>3</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H8" s="2" t="s">
         <v>17</v>
@@ -1080,7 +1103,7 @@
         <v>18</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="K8" s="2" t="s">
         <v>20</v>
@@ -1088,13 +1111,13 @@
     </row>
     <row r="9" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>14</v>
@@ -1103,10 +1126,10 @@
         <v>3</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H9" s="2" t="s">
         <v>17</v>
@@ -1114,8 +1137,8 @@
       <c r="I9" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="J9" s="4" t="s">
-        <v>40</v>
+      <c r="J9" s="3" t="s">
+        <v>54</v>
       </c>
       <c r="K9" s="2" t="s">
         <v>20</v>
@@ -1123,13 +1146,13 @@
     </row>
     <row r="10" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>14</v>
@@ -1138,10 +1161,10 @@
         <v>3</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H10" s="2" t="s">
         <v>17</v>
@@ -1150,7 +1173,7 @@
         <v>18</v>
       </c>
       <c r="J10" s="4" t="s">
-        <v>40</v>
+        <v>58</v>
       </c>
       <c r="K10" s="2" t="s">
         <v>20</v>
@@ -1158,13 +1181,13 @@
     </row>
     <row r="11" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>14</v>
@@ -1173,10 +1196,10 @@
         <v>3</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H11" s="2" t="s">
         <v>17</v>
@@ -1184,8 +1207,8 @@
       <c r="I11" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="J11" s="4" t="s">
-        <v>59</v>
+      <c r="J11" s="3" t="s">
+        <v>62</v>
       </c>
       <c r="K11" s="2" t="s">
         <v>20</v>
@@ -1193,13 +1216,13 @@
     </row>
     <row r="12" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>14</v>
@@ -1208,10 +1231,10 @@
         <v>4</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="H12" s="2" t="s">
         <v>17</v>
@@ -1219,8 +1242,8 @@
       <c r="I12" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="J12" s="4" t="s">
-        <v>65</v>
+      <c r="J12" s="5" t="s">
+        <v>68</v>
       </c>
       <c r="K12" s="2" t="s">
         <v>20</v>
@@ -1228,13 +1251,13 @@
     </row>
     <row r="13" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>14</v>
@@ -1243,10 +1266,10 @@
         <v>5</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="H13" s="2" t="s">
         <v>17</v>
@@ -1254,8 +1277,8 @@
       <c r="I13" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="J13" s="4" t="s">
-        <v>71</v>
+      <c r="J13" s="3" t="s">
+        <v>74</v>
       </c>
       <c r="K13" s="2" t="s">
         <v>20</v>
@@ -1263,13 +1286,13 @@
     </row>
     <row r="14" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>14</v>
@@ -1278,10 +1301,10 @@
         <v>5</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="H14" s="2" t="s">
         <v>17</v>
@@ -1289,8 +1312,8 @@
       <c r="I14" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="J14" s="4" t="s">
-        <v>40</v>
+      <c r="J14" s="5" t="s">
+        <v>79</v>
       </c>
       <c r="K14" s="2" t="s">
         <v>20</v>
@@ -1298,13 +1321,13 @@
     </row>
     <row r="15" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>14</v>
@@ -1313,10 +1336,10 @@
         <v>5</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="H15" s="2" t="s">
         <v>17</v>
@@ -1325,7 +1348,7 @@
         <v>18</v>
       </c>
       <c r="J15" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="K15" s="2" t="s">
         <v>20</v>
@@ -1333,13 +1356,13 @@
     </row>
     <row r="16" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>14</v>
@@ -1351,7 +1374,7 @@
         <v>24</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="H16" s="2" t="s">
         <v>17</v>
@@ -1359,8 +1382,8 @@
       <c r="I16" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="J16" s="4" t="s">
-        <v>40</v>
+      <c r="J16" s="3" t="s">
+        <v>88</v>
       </c>
       <c r="K16" s="2" t="s">
         <v>20</v>
@@ -1368,13 +1391,13 @@
     </row>
     <row r="17" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>14</v>
@@ -1383,10 +1406,10 @@
         <v>7</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="H17" s="2" t="s">
         <v>17</v>
@@ -1394,8 +1417,8 @@
       <c r="I17" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="J17" s="4" t="s">
-        <v>89</v>
+      <c r="J17" s="3" t="s">
+        <v>94</v>
       </c>
       <c r="K17" s="2" t="s">
         <v>20</v>
@@ -1403,25 +1426,25 @@
     </row>
     <row r="18" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E18" s="2">
         <v>8</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="H18" s="2" t="s">
         <v>17</v>
@@ -1438,16 +1461,16 @@
     </row>
     <row r="19" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="C19" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="D19" s="2" t="s">
         <v>98</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>93</v>
       </c>
       <c r="E19" s="2">
         <v>8</v>
@@ -1456,7 +1479,7 @@
         <v>24</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="H19" s="2" t="s">
         <v>17</v>
@@ -1473,16 +1496,16 @@
     </row>
     <row r="20" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E20" s="2">
         <v>8</v>
@@ -1491,7 +1514,7 @@
         <v>24</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="H20" s="2" t="s">
         <v>17</v>
@@ -1508,13 +1531,13 @@
     </row>
     <row r="21" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>14</v>
@@ -1526,7 +1549,7 @@
         <v>24</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="H21" s="2" t="s">
         <v>17</v>
@@ -1543,13 +1566,13 @@
     </row>
     <row r="22" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="D22" s="2" t="s">
         <v>14</v>
@@ -1561,7 +1584,7 @@
         <v>24</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="H22" s="2" t="s">
         <v>17</v>
@@ -1593,74 +1616,74 @@
     <col min="3" max="4" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
-        <v>110</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>111</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="D1" s="5" t="s">
+    <row r="1" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="D1" s="6" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="B2" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="C2" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="D2" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="B3" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="C3" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="D3" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="B4" t="s">
+        <v>125</v>
+      </c>
+      <c r="C4" t="s">
         <v>120</v>
       </c>
-      <c r="C4" t="s">
-        <v>115</v>
-      </c>
       <c r="D4" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>126</v>
+      </c>
+      <c r="B5" t="s">
+        <v>127</v>
+      </c>
+      <c r="C5" t="s">
+        <v>120</v>
+      </c>
+      <c r="D5" t="s">
         <v>121</v>
-      </c>
-      <c r="B5" t="s">
-        <v>122</v>
-      </c>
-      <c r="C5" t="s">
-        <v>115</v>
-      </c>
-      <c r="D5" t="s">
-        <v>116</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Dealer programme: D-3 closed (same cause as D-2); instant approval, commission and rating confirmed on staging
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/dealer-programme/DEALER_PROGRAMME_TRACKER_2026-10-28.xlsx
+++ b/docs/dealer-programme/DEALER_PROGRAMME_TRACKER_2026-10-28.xlsx
@@ -218,7 +218,7 @@
     <t>4500808, 6db91cd</t>
   </si>
   <si>
-    <t>FAIL — D-2 fixed in code, D-3 open</t>
+    <t>PASS — approved + e-mail; D-2 fixed in code</t>
   </si>
   <si>
     <t>GKS-CM-001</t>
@@ -251,7 +251,7 @@
     <t>22a74db, 9e3e1b7</t>
   </si>
   <si>
-    <t>FAIL — no accrual on staging (D-3)</t>
+    <t>PASS — ₹100 + ₹150 earned; payout not run</t>
   </si>
   <si>
     <t>GKS-CM-003</t>
@@ -263,7 +263,7 @@
     <t>Rating 0–10 by live shops (slabs), start rating, downgrade, bonus</t>
   </si>
   <si>
-    <t>PARTIAL — slabs visible; no accrual yet</t>
+    <t>PASS — activated shop counted</t>
   </si>
   <si>
     <t>GKS-DB-001</t>
@@ -418,7 +418,7 @@
       <b/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -440,11 +440,6 @@
         <fgColor rgb="FFFEF3C7"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFEE2E2"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -458,7 +453,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -470,9 +465,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1242,7 +1234,7 @@
       <c r="I12" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="J12" s="5" t="s">
+      <c r="J12" s="3" t="s">
         <v>68</v>
       </c>
       <c r="K12" s="2" t="s">
@@ -1312,7 +1304,7 @@
       <c r="I14" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="J14" s="5" t="s">
+      <c r="J14" s="3" t="s">
         <v>79</v>
       </c>
       <c r="K14" s="2" t="s">
@@ -1347,7 +1339,7 @@
       <c r="I15" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="J15" s="4" t="s">
+      <c r="J15" s="3" t="s">
         <v>83</v>
       </c>
       <c r="K15" s="2" t="s">
@@ -1616,17 +1608,17 @@
     <col min="3" max="4" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
+    <row r="1" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="5" t="s">
         <v>10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Dealer programme: released to production 28 Oct (flags off); report and tracker updated
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/dealer-programme/DEALER_PROGRAMME_TRACKER_2026-10-28.xlsx
+++ b/docs/dealer-programme/DEALER_PROGRAMME_TRACKER_2026-10-28.xlsx
@@ -74,7 +74,7 @@
     <t>PASS — incl. operator refused</t>
   </si>
   <si>
-    <t>Not released (flags off)</t>
+    <t>Released 28 Oct (ea7eecb, 8d6ef40) — flags off</t>
   </si>
   <si>
     <t>FEE-SLABS</t>
@@ -377,7 +377,7 @@
     <t>On, Pune only (28 Oct)</t>
   </si>
   <si>
-    <t>Off</t>
+    <t>Off (checked 28 Oct)</t>
   </si>
   <si>
     <t>gov_verification_auto_approval_enabled</t>

</xml_diff>